<commit_message>
doc(tables): fix dangling Breimann25a citation key -> Breimann25 in benchmarks table
Completes the Breimann25a -> Breimann25 rename (35cd4728): cells J14/J15 of
t1_overview_benchmarks.xlsx still referenced the old key, which broke the docs
build (missing reference in t1_overview_benchmarks). Repoint to [Breimann25].

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/source/index/tables/t1_overview_benchmarks.xlsx
+++ b/docs/source/index/tables/t1_overview_benchmarks.xlsx
@@ -922,7 +922,6 @@
       <c r="G11" t="n">
         <v>790</v>
       </c>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>Prediction of subcellular location of protein (cytoplasm vs plasma membrane)</t>
@@ -1059,7 +1058,6 @@
       <c r="G14" t="n">
         <v>63</v>
       </c>
-      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>Prediction of gamma-secretase substrates</t>
@@ -1067,7 +1065,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Breimann25a</t>
+          <t>Breimann25</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -1102,7 +1100,6 @@
       <c r="G15" t="n">
         <v>0</v>
       </c>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>Prediction of gamma-secretase substrates (PU dataset)</t>
@@ -1110,7 +1107,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Breimann25a</t>
+          <t>Breimann25</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">

</xml_diff>